<commit_message>
Daily news scrape: 2026-10-30
</commit_message>
<xml_diff>
--- a/EBRD.xlsx
+++ b/EBRD.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -3609,6 +3609,1093 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-supports-growth-of-auto-rubber-in-uzbekistan.html</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+The European Bank for Reconstruction and Development (EBRD) is helping to strengthen privately owned businesses in Uzbekistan by financing the expansion of a producer of automotive rubber products, Auto Rubber. The Bank is extending a loan of up to US$ 10 million (€8.8 million) to Auto Rubber, an established domestic manufacturer of automotive rubber sealing systems and other technical rubber components. The loan will finance the company’s development programme, as well as the expansion and localisation of its production facilities.
+The project will help to transform Auto Rubber into a diversified automotive component manufacturer by financing the installation of new equipment for the manufacture of semi-finished products, as well as a rubber-compound production line.
+The EBRD will support Auto Rubber in strengthening its corporate governance and advancing gender equality by helping it to adopt formal internal policies.
+The project is supported by grant funding from the Japan-EBRD Cooperation Fund.
+The EBRD has invested almost US$ 7.3 billion (€6.5 billion) in Uzbekistan to date through 219 projects, with most of those funds going to support private entrepreneurship.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:08:57.708609+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>EBRD extends loan to Star Group in Uzbekistan</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-extends-loan-to-star-group-in-uzbekistan.html</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+The European Bank for Reconstruction and Development (EBRD) is promoting entrepreneurial initiative and strengthening privately owned businesses in Uzbekistan by supporting the operations of consumer goods retailer Star Group.
+The EBRD is lending up to US$ 20 million (€17.7 million) to Support Samarqand, Bloomshop, Star Distribution and Star FMCG, collectively known as Star Group, a rapidly growing local distributor of fast-moving consumer goods.
+The loan will finance Star Group’s working capital needs and facilitate its business expansion, including that of its Tashkent- and Samarkand-based beauty-shop retail chain. The group will use the funds to both grow its regional presence and expand its product range.
+The project will also benefit from grant funding provided by the Bank and the Japan-EBRD Cooperation Fund to help Star Group to develop its corporate governance action plan.
+The EBRD will further help Star Group to support women’s careers and keep talented female staff by setting up a mentorship programme.
+The EBRD has invested almost US$ 7.3 billion (€6.5 billion) in Uzbekistan to date through 219 projects, with most of those funds going to support private entrepreneurship.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:00.170516+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>EBRD and GCF scale up support for greener cities</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-and-gcf-scale-up-support-for-greener-cities.html</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+The European Bank for Reconstruction and Development (EBRD) and the Green Climate Fund (GCF) are scaling up their partnership to support urban climate action, with the GCF approving a second €87 million financing tranche for the EBRD Green Cities programme.
+The new tranche doubles the amount of GCF concessional financing available for the programme to €174 million. It will help cities in eligible countries to address pressing climate mitigation and adaptation challenges through investment, policy support, capacity building and access to green finance.
+EBRD Green Cities has more than 60 participating cities and supports investment in sectors including urban transport, district energy, solid waste, renewable energy, smart solutions, water and wastewater, building, electricity distribution networks, street lighting, climate resilience and nature-based solutions.
+GCF concessional financing helps cities develop more ambitious investments while addressing affordability and bankability constraints, and mobilising additional public and private capital. It is available to cities, utilities and private-sector firms in 15 countries: Albania, Armenia, Bosnia and Herzegovina, Georgia, Jordan, Kazakhstan, the Kyrgyz Republic, Moldova, Mongolia, Morocco, North Macedonia, Serbia, Tajikistan, Tunisia and Uzbekistan.
+Support is provided through policy work, sustainable infrastructure investment, technical assistance and capacity building, and measures to improve access to green finance.
+The first tranche of GCF financing supported the completion of eight Green City Action Plans (GCAPs), the tailor-made strategies that help cities identify, prioritise and tackle their most pressing environmental challenges, and ten investments, including the River Bic Rehabilitation and Flood Protection project in Chisinau, Moldova – the first time the EBRD has formally implemented a nature-based solution as part of a project. The second tranche will enable the programme to expand its support for investments in participating cities.
+The approval comes as the EBRD and GCF approach 10 years of broader partnership and active project implementation. Over the past decade, the two institutions have worked together across a range of programmes and sectors to advance climate mitigation and adaptation, combining GCF concessional resources with EBRD financing, technical expertise and private-sector mobilisation. 
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:03.388014+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>EBRD and UniCredit Bank Banja Luka support energy-efficient businesses and buildings</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-and-unicredit-bank-banja-luka-support-energy-efficient-busi.html</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+Author: Bojana Vlajcic
+Businesses and housing developers in Bosnia and Herzegovina will be able to benefit from a new €9 million financing package for energy-efficient equipment, renewable energy and greener residential buildings.
+The European Bank for Reconstruction and Development (EBRD) is providing the funds to UniCredit Bank Banja Luka, which will lend the money to eligible businesses.
+Of the total, €5 million will be available to Small and Medium-sized Enterprises (SMEs) investing in energy-efficient and renewable-energy technologies. The funding is being provided under the SME Go Green programme. On successful completion, SMEs will be able to benefit from cashback incentives funded by the European Union (EU).
+A further €4 million, through the Western Balkans Green Economy Financing Facility (GEFF)*, will support investment in high-performance residential buildings and energy-efficiency and renewable energy measures in the residential sector. The programme aims to encourage more energy-efficient construction and lower-carbon building solutions to help households to benefit from lower energy consumption and reduced energy costs.
+Stela Melnic, EBRD Head of Bosnia and Herzegovina, said: “Reducing energy use in businesses and homes is part of Bosnia and Herzegovina’s transition to a lower-carbon economy. These loans will finance more efficient equipment, renewable energy and improvements to residential buildings, helping borrowers reduce their energy consumption and associated emissions.”
+Spas Vidarkinsky, CEO of UniCredit Bank Banja Luka, said: “At UniCredit, supporting the green transition means creating tangible benefits for our clients, communities and the wider economy. Through this partnership with the EBRD, we are providing businesses and residential developers with greater access to financing for investments that improve energy efficiency, accelerate the adoption of renewable energy and strengthen long-term competitiveness. As a bank committed to sustainable finance, we are proud to support Bosnia and Herzegovina’s journey towards a more resilient and lower-carbon future.“
+This financing further strengthens UniCredit Bank Banja Luka’s commitment to supporting the green transition of the domestic economy and promoting sustainable business models across all client segments.
+UniCredit Bank Banja Luka, first bank on Republic of Srpska market to offer EBRD lines SME Go Green and GEFF, is one of the leading banks in Republic of Srpska and part of UniCredit Group, one of Europe’s leading banking groups. Through its comprehensive range of retail and corporate banking services, the Bank actively supports sustainable growth, innovation and the transition towards a greener economy.
+The agreement reflects the long-standing cooperation between EBRD and UniCredit Bank Banja Luka in advancing sustainable finance and supporting investments that generate positive environmental and economic impact.
+The EBRD has invested more than €3.4 billion in Bosnia and Herzegovina to date, with a strong focus on supporting private-sector competitiveness, green transition and sustainable infrastructure development.
+*The EBRD’s GEFF programme in the Western Balkans is co-funded by the EU through the Western Balkans Investment Framework, Austria, Denmark, Japan, and Austria and Switzerland through the High-Impact Partnership on Climate Action (HIPCA)**.
+**The EBRD’s HIPCA is supported by Austria, Canada, Finland, Germany, the Netherlands, the Republic of Korea, Spain, Switzerland, TaiwanICDF, the United Kingdom, and the United States of America.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:06.495552+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>EBRD and EU expand finance for small businesses in Montenegro</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-and-eu-expand-finance-for-small-businesses-in-montenegro.html</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+The European Bank for Reconstruction and Development (EBRD) is providing a €10 million financing package to Alter Modus, Montenegro’s leading microfinance institution, to improve access to finance for micro, small and medium-sized enterprises (MSMEs), including businesses led by women and young entrepreneurs.
+The package comprises a €7 million loan for MSMEs, a €2 million loan under the Western Balkans Women in Business programme and a €1 million loan under the Western Balkans Youth in Business programme. This will enable Alter Modus to increase lending to private businesses across Montenegro, including firms outside the capital, Podgorica.
+The Women in Business loan will expand access to finance for women-led MSMEs, while the Youth in Business loan will support MSMEs owned or led by entrepreneurs under the age of 35.
+The European Union (EU) is supporting the Women in Business and Youth in Business loans through the European Fund for Sustainable Development Plus (EFSD+), providing first-loss risk cover and programme-level technical assistance. In addition to the EU, those two loans are also being supported by Luxembourg and Italy through the Central European Initiative.
+The €7 million MSME loan will finance eligible private enterprises’ investment and expansion needs in Montenegro. At least 20 per cent of this financing is expected to support green investment, including improvements in energy and resource efficiency.
+Ekaterina Solovova, the EBRD’s Head of Montenegro, said: “Micro, small and medium-sized enterprises are a key driver of Montenegro’s economy, creating jobs and supporting growth across the country. Through this financing package, we are improving access to finance for businesses that continue to face barriers to funding, particularly women-led and youth-led enterprises. Our longstanding partnership with Alter Modus and the support of the European Union will help entrepreneurs to invest, grow and create new opportunities in communities throughout Montenegro.”
+Ana Kentera, the CEO of Alter Modus, said: “Our continued partnership with the EBRD allows us to reach more businesses across Montenegro and provide financing where it is needed most. This new €10 million package will help us better support small businesses, particularly those led by women and young entrepreneurs, as they grow and explore more sustainable business solutions. Together with our international partners, we remain committed to making financing more accessible and providing long-term support for our clients’ entrepreneurial ventures.”
+Bernard Brunet, Head of Cooperation at the Delegation of the European Union to Montenegro, said: “The development of new, innovative companies is crucial for sustainable economic development in Montenegro, and will ensure that the country can take full advantage of the EU Single Market after accession. The guarantees provided by the European Union to the EBRD will ensure that Alter Modus can offer financial support package at competitive conditions and for clients who might otherwise face more constraints to access financial resources for developing their projects.”
+Alter Modus, one of the country’s leading microfinance institutions, is a longstanding EBRD partner, having worked with the Bank in Montenegro since 2004.
+The EBRD is a leading institutional investor in Montenegro, having invested €1.1 billion across 116 projects to date. Its investments support the country’s sustainable development, infrastructure, private-sector growth and regional integration.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:09.545822+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>EBRD supports expansion of automotive production in Bosnia and Herzegovina</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-backs-car-production-growth-in-bosnia-and-herzegovina.html</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+The European Bank for Reconstruction and Development (EBRD) is providing a €15 million loan to Selzer Automotive Bosnia, a manufacturer of ready-to-install metal components and assemblies for the automotive industry.
+The investment will finance new machinery, tools and production equipment at the company’s plant in Bosnia and Herzegovina. Most of the initial loan will support the production of components for electric and low-emission hybrid vehicles, including rotor shafts used in electric motors and components for hybrid-vehicle transmissions.
+The project will help Selzer Automotive Bosnia expand production, improve its operational performance and strengthen its integration into European automotive supply chains. The company manufactures precision metal components and assemblies for automotive transmissions, brakes and engines, supplying major international automotive manufacturers and Tier 1 suppliers.
+The EBRD will also support the company’s workforce development. The project envisages training and employment opportunities for at least 100 additional workers, with a focus on young people and women. Planned measures include establishing structured training for computer numerical control (CNC) and automated process operators, developing cooperation with vocational schools and strengthening equal-opportunity employment practices.
+Stela Melnic, EBRD Head of Bosnia and Herzegovina, said: “This investment supports the continued development of Bosnia and Herzegovina’s manufacturing sector and its closer integration into European value chains. By helping Selzer Automotive Bosnia expand production of components for electric and low-emission vehicles, we are supporting a more competitive and greener economy. Just as importantly, the project will invest in people by developing technical skills and creating new employment opportunities, particularly for young people and women.”
+Michael Stötzel, Chief Executive Officer of Selzer Group, said: “The EBRD’s financing of €15 million is a strong vote of confidence in the Selzer Group and the future of our operations in Bosnia and Herzegovina. It enables us to invest in new machinery, advanced manufacturing technologies and increased production capacity for electric and hybrid vehicle components. This investment will strengthen our competitiveness, help secure local jobs over the long term and lay the foundation for further investment and growth.”
+“For me, it is particularly important that this development also provides a long-term perspective for our employees,” he continued. “Through targeted training and the development of young talent, we aim to strengthen local expertise and create new career opportunities. We thank the EBRD for its trust and partnership in supporting the continued development of our operations in Bosnia and Herzegovina.”
+Selzer Automotive Bosnia is part of the Selzer Group, a German automotive industrial group that develops and produces metal components and assemblies for automotive transmissions, brakes and engines, as well as industrial applications. The group has operated in Bosnia and Herzegovina since 2021 and is owned by German investment company Mutares.
+The investment is aligned with the EBRD’s priorities in Bosnia and Herzegovina by supporting private-sector competitiveness, workforce skills and the transition towards lower-carbon technologies.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:12.020449+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>EBRD and GCF launch Uzbekistan GEFF Greening Financial Systems framework</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-and-gcf-launch-uzbekistan-geff-greening-financial-systems-f.html</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+Author: Anton Usov
+The European Bank for Reconstruction and Development (EBRD) and the Green Climate Fund (GCF) are encouraging more households and businesses in Uzbekistan to invest in green and innovative technologies by launching the next phase of the Green Economy Financing Facility (GEFF), the Greening Financial Systems (GFS) framework, in the country. The GFS will support investments that promote the efficient use of water, sustainable land management and greater resource efficiency.
+Hamkorbank, Uzbekistan’s third-largest lender, will receive a financing package of up to US$ 20 million (€17.8million) under the GFS and will become the first local bank to join the framework. It will use the funds (available in synthetic Uzbek som or in US dollars) to support private-sector investments in climate change mitigation (such as energy-efficiency measures) and adaptation (such as agricultural irrigation) across the country.
+The package consists of an EBRD loan of up to US$ 18 million (€16 million) and GCF concessional financing of up to US$ 2 million (€1.8 million). Potential projects supported through this financing could facilitate a reduction in CO2 emissions of around 5,685 tonnes a year.
+The GEFF GFS programme in Uzbekistan will build upon the EBRD's GEFF I and GEFF II, which have together established a financing framework of US$ 160 million for green investments since their launch in 2018 and 2023, respectively. GEFF has supported 425 green projects in the country through five participating financial institutions, helping large companies and small and medium-sized enterprises gain access to climate technologies ranging from energy-efficient equipment and electric vehicles to solar photovoltaic systems and industrial decarbonisation solutions. Close to 10 per cent of projects have supported women-led or owned businesses.
+GEFF in Uzbekistan has delivered annual energy savings of approximately 1.1 million GJ and helped to reduce annual CO2 emissions by around 53,000 tonnes. It has also supported the creation of more than 14.3 MW of renewable energy capacity and helped to strengthen the green finance capabilities of local financial institutions.
+The GEFF GFS programme will work to scale up climate finance and promote the transition of Uzbekistan’s financial sector towards climate-aligned lending and investment practices.
+The EBRD has invested almost US$ 6.9 billion (€6.1 billion) in Uzbekistan through 217 projects, with most of the funds supporting private entrepreneurship.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:15.154782+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>EBRD supports youth entrepreneurship in Uzbekistan</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-supports-youth-entrepreneurship-in-uzbekistan.html</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+More young entrepreneurs in Uzbekistan will benefit from Davr Bank expanding its lending under the European Bank for Reconstruction and Development (EBRD) Youth in Business (YiB) programme for Central Asia, targeting micro, small and medium-sized enterprises (MSMEs) that are led or owned by individuals under the age of 35.
+A senior EBRD loan of up to US$ 25 million (€22 million) under the YiB will be disbursed either in synthetic Uzbek som or in US dollars. At least one third of these funds will be channelled towards women-led MSMEs. Davr Bank will also target MSMEs based in rural areas of Uzbekistan.
+Eligible young clients of Davr Bank will benefit from training, advisory support and other non-financial services provided under the EBRD’s Advice for Small Businesses programme.
+According to government data, more than 26 per cent of Uzbekistan’s population is aged 30 or under. This young generation represents a dynamic, technically and digitally skilled workforce that will need new job opportunities in the coming years. Creating these opportunities is one of the EBRD’s priorities.
+The project will also support greater outreach to youth-led MSMEs outside the capital and help Davr Bank further develop its systems and products for serving young entrepreneurs.
+The EBRD has invested almost US$ 7.3 billion (€6.5 billion) in Uzbekistan to date through 219 projects, with most of those funds going to support private entrepreneurship.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:19.303482+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>The difference clean, reliable water makes</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/videos/2026/the-difference-clean--reliable-water-makes.html</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>The difference clean, reliable water makes
+Surrounded by mountains and close to the shores of Lake Issyk-Kul, Karakol in the Kyrgyz Republic is known for its natural beauty, relaxed pace of life and growing tourism sector. But behind the city's picturesque setting, access to reliable drinking water has long been a challenge.
+For some residents, water shortages were simply part of everyday life. "Sometimes we had to wake up at four in the morning just to fill containers," recalls Valentina, a Karakol resident. "There was no running water inside the house."
+Much of the city's water infrastructure was built decades ago. Ageing pipelines and interruptions in supply made even simple daily activities, from cooking and cleaning to running a small business, more difficult.
+Today, that is changing.
+With financing from the European Bank for Reconstruction and Development (EBRD) and grant support from Switzerland, through the State Secretariat for Economic Affairs (SECO), Karakol is modernising its water supply system.
+“Clean water is essential to our lives. From the moment we wake up, we need it.” — Albina, resident of Karakol
+The investment is helping the municipal water utility, Karakol Vodokanal, replace ageing pipelines, upgrade water facilities and introduce water meters to improve efficiency and encourage more responsible consumption.
+For residents in neighbourhoods where the networks have already been upgraded, the difference is tangible. "Now there's no need to store water in containers," says Valentina. "You simply turn on the tap and the water is there."
+Reliable water also matters for Karakol's local economy. Guesthouses, hotels and other small businesses depend on clean water to welcome visitors and provide quality services. For Nao, who runs a guesthouse in the city, improvements in water supply have made it easier to look after her guests.
+Select an image to expand
+Select an image to expand
+The project is not only about bringing water into homes and businesses. It is also about making better use of a precious natural resource. "Water is not endless," explains Olga, who works on the project at Karakol Vodokanal. "We want even children to understand the importance of turning off the tap."
+As Karakol continues to develop, modern and efficient water infrastructure will be essential to supporting its residents, local businesses and more sustainable use of resources.
+Video for media use
+If you would like a broadcast-quality version of this or any other EBRD video, including B-roll, please contact our Communications Department.</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:22.551971+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>EBRD and EU launch Green Economy Financing Facility to support the Palestinian economy</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-and-eu-launch-palestinian-green-financing-facility.html</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+The European Bank for Reconstruction and Development (EBRD) and the European Union (EU) launched the Green Economy Financing Facility (GEFF) to support the Palestinian economy, expanding access to finance for green investments that will help businesses and households lower costs, improve competitiveness and strengthen climate resilience.
+The programme will support investments in renewable energy, energy and resource efficiency, green buildings, circular economy solutions and waste management, helping businesses and households lower costs, improve competitiveness and strengthen climate resilience.
+Through a €25.9 million financing facility, the EBRD is working with local partner financial institutions to increase access to green finance. The programme combines EBRD financing with technical expertise and EU-funded investment incentives of up to 25 per cent to households and businesses for eligible and verified investments, helping accelerate the adoption of high-performance green technologies across the Palestinian economy.
+The facility also aims at improving access to green finance for women and women-led businesses. Dedicated technical assistance and capacity-building activities will support participating financial institutions, households and businessesthroughout the programme.
+GEFF-supported investments are expected to deliver significant environmental benefits. The investments done under the programme to date are already expected to generate annual savings of 12,656 MWh of primary energy and avoid 3,717 tonnes of carbon dioxide emissions, while reducing water consumption and waste generation.
+Since the start of its activities in the West Bank and Gaza in 2017, the EBRD has approved 42 projects worth a total of €225 million.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:32.823518+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>A modern kitchen, powered by the sun</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/videos/2026/a-modern-kitchen--powered-by-the-sun.html</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>A modern kitchen powered by the sun
+At KumKuma, sunshine is helping power the kitchen, bringing modern Armenian flavours to the table with lower energy costs and a smaller carbon footprint.
+At KumKuma restaurant in Gyumri, modern Armenian dishes come with a secret ingredient: sunshine. A rooftop solar system is helping power the restaurant’s busy kitchen, cutting energy costs and reducing its carbon footprint.
+The investment was financed through Inecobank under the EU4Business-EBRD Credit Line, with EU-funded grant support and expert technical guidance helping the restaurant make the switch to solar.
+KumKuma is one of hundreds of businesses across Armenia supported by the EBRD and the European Union (EU) to invest in modern technologies, improve efficiency and grow more sustainably.</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:35.949945+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>EBRD President Odile Renaud-Basso to visit Montenegro</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-president-odile-renaud-basso-to-visit-montenegro.html</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+The President of the European Bank for Reconstruction and Development (EBRD), Odile Renaud-Basso, will visit Montenegro this week to participate in the Berlin Process Leaders' Summit in Sveti Stefan. She will speak at the summit and hold a number of bilateral meetings with national and institutional leaders on the margins. Later, in Podgorica, she will hold a series of meetings with senior Montenegrin government officials, development partners, clients and representatives of the business and diplomatic communities.
+The EBRD strongly supports the key objectives of the Berlin Process, including furthering regional integration in the Western Balkans and gradually integrating it into the EU. The Bank is a leader in funding the Western Balkans connectivity agenda and the largest international financial institution investor in the Western Balkans. In 2025 alone, it invested €1.7 billion in the region. The Bank has more than 160 staff on the ground, located in six Resident Offices and a growing regional hub.
+President Renaud-Basso’s visit to Montenegro comes at an important moment in the country's development as it advances its EU accession agenda and pursues major investments in sustainable infrastructure, connectivity and energy security. During her meetings, the EBRD President will discuss how the EBRD can continue to support Montenegro's reform priorities and economic development through investments, policy engagement and technical assistance.
+Ahead of the visit, President Renaud-Basso said: “Montenegro has made important progress on its European path and has a real opportunity to translate this momentum into lasting economic gains for its citizens. The EBRD remains a committed partner to Montenegro, supporting investments and reforms that strengthen competitiveness, accelerate the green transition and improve connectivity. I look forward to discussing with our partners how we can continue to work together to support sustainable growth and the country's EU aspirations.”
+Montenegro is one of the most advanced EU accession candidates in the Western Balkans. The EBRD has invested more than €1.1 billion in the country to date through projects that support greener, more resilient and more inclusive economic growth. Recent investments include financing for intelligent transport systems, railway modernisation and renewable energy development.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:40.348998+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Early Market Engagement (EME) for the Port of Cotonou Project - 10 Nov</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/events/early-market-engagement--eme--for-the-port-of-cotonou-project.html</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Early Market Engagement (EME) for the Port of Cotonou Project
+Event details
+The European Bank for Reconstruction and Development invites you to an upcoming Early Market Engagement webinar for the Port of Cotonou Project in Benin.
+The EME aims to provide interested companies, contractors, consultants and other market participants with early visibility of upcoming procurement opportunities under the Project and an opportunity to learn more about the anticipated requirements ahead of the formal procurement processes.
+The Project will support the safe, efficient and sustainable operation of the Port of Cotonou through the development and rehabilitation of critical operational infrastructure assets. The Project is expected to contribute to improved operational efficiency, workforce professionalisation, institutional strengthening and environmental sustainability at one of Benin's most important economic assets, the Port of Cotonou.
+Through this Early Market Engagement, the EBRD and PAC intend to engage with the market at an early stage, raise awareness of the forthcoming opportunities and encourage strong market interest in the future EBRD-financed procurement processes.
+Interested companies are encouraged to participate in the EME and familiarise themselves with the Project and the anticipated procurement opportunities.
+Participation in the EME does not form part of any subsequent procurement process and does not confer any advantage or preferential treatment in future tenders.
+Further information on the Port of Cotonou Project is available on the EBRD Project 56249 page.</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:54.639842+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>EBRD backs largest solar PV project in Egypt and Africa</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-backs-largest-solar-pv-project-in-egypt-and-africa.html</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+The European Bank for Reconstruction and Development (EBRD) is strengthening Egypt’s renewable energy capacity and energy security by helping to finance a new large-scale solar power plant and battery energy storage system (BESS) in Minya. The facility is set to become the largest solar power plant in Egypt and Africa, with a capacity of 1.2 GW.
+The Bank is arranging a loan of up to US$ 265 million (€232 million) to Nefer Menya for Renewable Energy S.A.E. (Nefer Menya), a special purpose vehicle owned by Infinity Power and HAU Energy B.V. The funding will consist of a US$ 160 million (€140.1 million) A-loan from the EBRD’s own funds, a US$ 75 million (€65.7 million) B-loan mobilised from Bank of Jordan and up to US$ 30 million (€26.3 million) in concessional financing from the CIF Clean Technology Fund (CTF) under its Global Energy Storage Program.
+Nefer Menya is being co-financed by German development finance institution DEG, the Dutch Entrepreneurial Development Bank (FMO) and France’s Proparco as part of an aggregate debt financing package of up to US$ 566 million (€494.7 million).
+The funds to Nefer Menya will be used for the construction and operation of a 1.2 GW solar power plant with a 600 MWh BESS, one of Egypt’s first projects to combine large-scale solar generation with battery storage. The battery system will store solar power generated during the day for use during peak demand after sunset, helping to strengthen grid stability and reliability.
+Electricity will be sold to the Egyptian Electricity Transmission Company under a 25-year power purchase agreement, providing clean, renewable power at a lower cost than conventional generation. The project is expected to avoid more than 1.5 million tonnes of CO2 emissions per year and to power more than 1.4 million homes.
+The investment supports the EBRD-led Energy Pillar of Egypt’s flagship Nexus of Water, Food and Energy, launched at COP27. The initiative aims to facilitate 10 GW of new private-sector renewable energy capacity while cutting 5 GW of inefficient fossil-fuel capacity.
+Infinity Power, a joint venture established in 2019 by Infinity and Masdar, is Africa’s largest pure-play renewable energy provider. The EBRD holds an equity stake in Infinity Power. HAU Energy B.V. was established in 2024 to develop renewable energy projects in Egypt and is owned by Meridiam, Hassan Allam Utilities and the EBRD.
+In addition to the concessional loan, the CTF will provide technical cooperation funding to introduce two nationally accredited technical training programmes focused on green skills for young labour-market entrants in Minya governorate, equipping them with future-ready skills and enhancing their employability in Egypt’s growing renewable energy sector. The CTF funding will also help Hassan Allam Utilities to strengthen its human resources policies and practices, embed gender equality into its workforce management strategy and enhance women’s access to technical and leadership roles in the traditionally male-dominated energy sector.
+Aida Sitdikova, EBRD Director of Sustainable Infrastructure in the Middle East and Africa, said: “The EBRD is proud to lead the financing of this landmark 1.2 GW solar PV and 600 MWh battery storage project, the largest in Egypt and Africa to date. Egypt continues to be a trailblazer in large-scale renewable energy deployment at affordable prices. By combining solar generation with utility-scale battery storage, this project will strengthen the country’s energy security and enhance grid resilience. We are delighted to partner once again with Infinity Power and Hassan Allam Utilities to support Egypt’s ambitious energy transition goals.”
+Samer Mirai, Regional Head of Corpoate Banking and Syndications of Bank of Jordan, said: “The Bank is proud to partner with the EBRD in financing this landmark renewable energy project, an important step in advancing Egypt’s energy transition and strengthening energy security. Our participation as both a B-loan lender and original hedge counterparty reflects our strong partnership with the EBRD and our growing role in supporting strategic, large-scale sustainable infrastructure across the region. The transaction is closely aligned with Bank of Jordan’s sustainability and green finance strategy, and reinforces our commitment to mobilising capital towards projects that contribute to a more sustainable and resilient energy future.”
+Eng. Nayer Fouad, Co-Founder and CEO of Infinity Power, said: “This landmark financing reflects strong confidence in Egypt’s renewable energy sector and Infinity Power’s ability to deliver large-scale clean energy infrastructure. As the largest solar PV project in Egypt and Africa, paired with one of the country’s first utility-scale battery energy storage systems, Nefer Menya will strengthen energy security, enhance grid resilience and support Egypt’s transition to a low-carbon economy. Together with HAU Energy and our financing partners, we are proud to deliver this flagship project as we advance towards our goal of 10 GW of operational renewable energy capacity by 2032 and expand access to affordable, reliable clean energy across Africa.”
+Dalia Wahba, CEO of Hassan Allam Utilities, said: “Securing this financing package shows what strong partnerships can achieve in mobilising capital for transformative energy infrastructure. Egypt has set a clear ambition to generate 42 per cent of its electricity from renewable sources by 2030, and Hassan Allam Utilities is committed to helping drive that agenda by delivering green, reliable infrastructure across the country. Through HAU Energy, alongside Infinity Power and our financing partners, we are combining large-scale solar generation with battery storage to provide clean power that is available when the grid needs it most. Every megawatt-hour we produce reduces reliance on imported fuel, strengthens Egypt’s energy security and builds a more competitive foundation for sustainable growth.”
+The EBRD is a leading institutional investor in Egypt. Since starting operations there in 2012, it has invested more than €16 billion through 238 projects.</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:09:57.368390+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>The EBRD at Biodiversity COP17 - 19 Oct</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/events/the-ebrd-at-biodiversity-cop17.html</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>The EBRD at Biodiversity COP17
+Event details
+The European Bank for Reconstruction and Development (EBRD) will take part in the 17th meeting of the Conference of the Parties to the Convention on Biological Diversity (COP17), reaffirming its commitment to supporting global efforts to halt and reverse biodiversity loss and translate international biodiversity goals into investment and action.
+The conference comes at an important moment for the implementation of the Kunming-Montreal Global Biodiversity Framework, as countries undertake the first global review of collective progress since the framework was adopted in 2022. COP17 will bring together governments, international organisations, development partners, businesses and civil society to advance the global biodiversity agenda.
+For the EBRD, protecting and restoring nature is closely linked to economic resilience and sustainable growth. Healthy ecosystems underpin food and water security, resilient infrastructure and supply chains, while biodiversity loss can create significant risks for economies and businesses.
+As a multilateral development bank (MDB) with a strong focus on private-sector investment, the EBRD brings together project origination, private-sector mobilisation, blended finance, policy dialogue, technical assistance and strong environmental and social safeguards.
+The EBRD delegation will be headed by Fatoumata Bouaré, Vice President and Chief Risk Officer, and will include senior representatives such as Gianpiero Nacci, Managing Director for Climate Strategy and Delivery, Maya Hennerkes, Managing Director for Environment and Sustainability, Elisabetta Falcetti, Managing Director for Türkiye and the Caucasus, and others who work across nature, climate, agribusiness and environmental and social sustainability.
+The EBRD will lead the following key events:
+- From restoration to investment: who pays for nature at scale?
+22 October | 10.00-11.00, Joint MDB pavilion and live here
+This event will bring together governments, private investors, project developers and MDBs to examine the business models, funding mechanisms and risk-sharing arrangements that can make restoration commercially viable. The discussion will focus on how restoration projects can generate sustainable revenue through mechanisms such as payments for ecosystem services, resilient agricultural and forestry value chains, biodiversity and carbon markets, water-related revenues and outcome-based public incentive schemes.
+Speakers will explore how public funding, philanthropy, concessional capital and MDB support can catalyse private investment, address residual risks and create investable portfolios that deliver measurable benefits for nature while enhancing economic resilience, strategic autonomy and long-term prosperity.
+- Building bridges: linking nature outcomes to infrastructure investment
+22 October | 15.00-16.15, Joint MDB pavilion and live here
+Infrastructure investments are one of the largest drivers of biodiversity loss, but they can also be among the most important supporters of biodiversity recovery. MDBs are increasingly testing different approaches to deliver nature-positive outcomes through infrastructure investments across agriculture, transport, energy, water and wastewater, coastal and marine infrastructure, the built environment and urban areas.
+Drawing on their practical experiences across sectors and regions, MDBs and their partners will use this session to explain how they are integrating nature into infrastructure planning, design, financing and long-term stewardship, and what it will take to move from individual or small-scale pilots to mainstreamed nature investment approaches. The discussion will focus not only on project-level success stories, but also on the governance, financing, monitoring and institutional arrangements required to sustain nature outcomes over time.
+- MDB nature finance – contributions to the implementation of the GBF
+26 October | 11.30-12.30, Vayk – Side-event Room 3 Side Event
+At the event, the MDB Nature Group will launch Common Principles, Taxonomy and Metrics: a voluntary high-level status report. The report represents a collaborative effort to publish MDBs’ progress on the application of the Common Principles, Nature Finance Taxonomy and Guidance on Results Metrics. It captures high-level information on the methodology, areas of focus, and early insights from initial implementation.
+- Compatibility of 30x30 and tripling renewable energy
+26 October | 13.15-14.30, Lori – Meeting Room 4 – Block 2, 3rd Floor Side Event
+This discussion will explore how policy support, integrated spatial planning, safeguards and good practice can help transform potential trade-offs into opportunities for nature-positive renewable energy development. Discussions will focus on practical experiences, lessons learned and innovative approaches for aligning climate and nature finance, reducing land-use conflicts, supporting ecosystem restoration and mobilising investment that delivers measurable benefits for both biodiversity and the energy transition.
+The event will provide a platform for identifying pathways to scale integrated climate and nature solutions and strengthen collaboration towards achieving global biodiversity and decarbonisation targets.
+- Financing the agrifood transition
+28 October | 10.00-11.00, Joint MDB pavilion and live here
+Mounting evidence shows that agricultural practices that conserve or restore the natural systems on which food production relies can be immediately low cost, and even profit-enhancing in the medium and long term. However, the agricultural transition has been slow to advance. Can finance help to accelerate its pace? What products and transactional structures do investors or corporates have available to target improved outcomes? What outcomes should be targeted? And what inputs, outputs or outcomes can and should be monitored across different time horizons, and by whom?
+This panel seeks to address these questions in conversation with multiple players in the financial ecosystem, based on their own experiences and new innovations.
+- Launch of MDB Briefing Note: Identifying opportunities to support biodiversity objectives through MDB operations
+28 October | 15.00-16.00, Joint MDB pavilion and live here
+This event will mark the launch of MDB Briefing Note: Identifying opportunities to support biodiversity objectives through MDB operations. Developed by the EBRD together with other MDBs, the briefing note explores the integration of biodiversity gains into development finance and identifies opportunities for nature recovery through established safeguarding approaches.
+The event will bring together MDBs, policymakers, conservation organisations and practitioners to discuss how biodiversity gains approaches can contribute to delivery of the Global Biodiversity Framework, mobilise investment for ecosystem restoration and scale nature-positive infrastructure across regions and sectors.</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:10:04.491673+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>MDB heads strengthen joint action in Manila to deliver more financing and greater impact</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/mdb-heads-strengthen-joint-action-in-manila-to-deliver-more-fina.html</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+The Heads of Multilateral Development Banks (MDBs) Group met at the Asian Development Bank (ADB) headquarters in Manila today to discuss how to deliver more financing and greater impact to support developing members as they face mounting challenges. It was the Group’s first-ever meeting in the Philippines, hosted by ADB as its 2026 Chair.
+“Conflict, economic uncertainty, high debt, inflation and disasters are placing growing pressure on our members and making development harder,” said ADB President Masato Kanda, host and current Chair of the MDB Heads Group. “Our meeting in Manila was an opportunity to turn shared commitments into practical action, so we can help members protect their development gains, attract investment, and build more resilient economies.”
+Against a backdrop of disasters, conflicts, difficult macroeconomic conditions, and constrained fiscal space, the Heads reaffirmed MDBs’ readiness to provide timely financial and analytical support to protect vulnerable populations and sustain investment in jobs and resilient long-term growth.
+In a joint statement, the Heads welcomed the significant progress achieved this year working as a system to mobilize private capital, and on joint actions to advance jobs, nature, climate, water, critical minerals, artificial intelligence and other common development priorities, and on efforts to enhance system efficiency for greater impact at scale, in line with each institution’s mandate, strategy and operational model.
+The role of Chair of the Heads of MDBs Group will be passed in December from ADB to the European Investment Bank Group.
+The Heads of MDBs Group includes the African Development Bank Group, Asian Development Bank, Asian Infrastructure Investment Bank, Council of Europe Development Bank, European Bank for Reconstruction and Development, European Investment Bank Group, Inter-American Development Bank Group, Islamic Development Bank, New Development Bank, and the World Bank Group. The International Monetary Fund also participates in the Heads discussions.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:10:08.401521+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>MDB collaboration framework citical minerals-to-manufacturing value chains</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/mdb-collaboration-framework-citical-minerals-to-manufacturing-va.html</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Multilateral Development Banks (MDBs) establish this Collaboration Framework to strengthen collective support for developing countries seeking to develop resilient, responsible, and diversified critical minerals-to-manufacturing value chains. The Framework responds to the need for coordinated action across policy and governance, environmental and social performance, enabling infrastructure, regional integration, project preparation, financing, market development, and learning. Its overarching purpose is to support countries translate mineral endowments into sustainable development outcomes while recognizing the foundational role of critical minerals value chains in the low-carbon transition.
+This includes more and better jobs, stronger institutions, local economic diversification, domestic value addition, regional trade, the deployment of clean-energy technologies, circular material flows and sustainable industrial development, and competitive participation in global supply chains.
+The Framework builds on the commitment made in the Joint MDB Statement on Critical Minerals to Manufacturing Value Chains issued on April 16, 2026. It recognizes that critical mineral value chains are complex systems extending from geological knowledge, exploration and mining to processing, refining, manufacturing, recycling, and enabling services. Their development requires coherent public policy, strong environmental and social performance, fit-for-purpose infrastructure, investable projects, long-term capital, and transparent and resilient markets.
+Implementation will be country-driven, development-focused, voluntary, flexible, and additional to existing bilateral or multilateral cooperation. Participating MDBs will collaborate where doing so improves development impact, efficiency, scale, or quality, subject to each MDB’s mandate, policies, approvals and available resources. Collaboration may involve all participating MDBs or smaller groups of interested institutions, depending on regional presence, sector expertise, financing instruments, and the needs of supported countries.1
+The framework will be implemented in three areas to advance efficiency, impact and sustainability of MDB engagement:
+The framework is composed of four high-level objectives, to be advanced over time through activities and deliverables identified each year. The MDB Working Group on Critical Minerals Value Chains will coordinate implementation under each objective and report annually to the Heads of MDBs Group on progress made.
+MDBs will advance practical cooperation on environmental and social requirements applicable to metals and minerals related activities with a focus on mining. The objective is to identify areas of convergence, promote mining-relevant good international industry practice (GIIP), best practices for mid- and downstream processing and manufacturing, and expand mutual reliance where institutional frameworks permit.
+Collaboration may include technical exchange on sector guidance; identification of appropriate mining, processing and manufacturing environmental, health, and safety practices; sector-specific requirements and due-diligence and monitoring, good practices and lessons learned; stronger coordination and alignment on sector-specific E&amp;S risks in mine planning, stakeholder engagement, grievance management, community benefits, indigenous people, biodiversity and ecosystem services, water and groundwater management, tailings management, pollution control, labor, occupational and community health and safety, land rights and resettlement, cumulative impacts, and mine closure among others; and use of existing or future mutual-reliance arrangements. For jointly supported operations, MDBs will seek proportionate and efficient approaches that maintain high standards while reducing avoidable duplication for supported countries.
+The intended result is stronger and more consistent client environmental and social performance, greater clarity for governments and sponsors, more efficient preparation and monitoring of joint operations, and increased confidence that projects supported by multiple MDBs meet robust requirements and consultation processes, including with local communities, civil society organizations (CSOs) and relevant non-governmental organizations (NGOs).
+MDBs will improve coordination of upstream advice, technical assistance, analytics, investment planning, and financing in countries and regions where several institutions are active. Country-level task teams will be established to exchange information, identify complementarities, reduce repeated diagnostics, align sequencing around government priorities, connect policy reform with infrastructure, industrialization and investment, and improve the technical human capacity needed across critical minerals-to-manufacturing value chains.
+Particular attention will be given to mineral corridors and associated systems—power, transport, logistics, water, digital connectivity, processing and manufacturing hubs, industrial zones, ports, and trade facilitation—as well as upstream mining investments, including opportunities across the mining project cycle. Recognizing the interdependence between bankable mining projects and the infrastructure and value chains they support, MDBs will identify opportunities for joint preparation, parallel financing, co-financing, guarantees, and coordinated technical assistance where collaboration can improve scale, bankability, or development impact. Regional engagement will address cross-border infrastructure, shared processing potential, market access, regulatory interoperability, customs and trade arrangements, and cooperation with regional bodies.
+The intended result is more coherent and sequenced support, integrated infrastructure and value-chain development, fewer gaps and overlaps, and stronger links between mineral production, domestic value addition, regional integration, new and better-quality jobs, industrialization, and broader economic transformation.
+MDBs work together to address the risks and financing constraints that limit investment across exploration, extraction, enabling infrastructure, processing, refining, manufacturing, and recycling. Collaboration focuses on stronger project preparation to provide risk mitigation tools related to coordinated engagement with governments and sponsors, appropriate risk allocation long-term and patient capital, guarantees and insurance, blended or concessional finance where justified, and innovative instruments suited to early-stage, large-scale, or market-constrained investments.
+MDBs may develop or participate in investment facilitation platforms, joint mandates, risk-sharing arrangements, offtake-linked financing, first-loss or cost-overrun facilities, early-stage equity vehicles, or other solutions consistent with their mandates. They will also convene producers, original equipment manufacturers, technology providers, infrastructure developers, investors, traders, and downstream users to clarify demand, technical requirements, supply-chain constraints, and bankability conditions.
+The intended result is a larger pipeline of well-prepared, high-standard investments; improved access to long-term finance; stronger market signals; more effective use of public and concessional resources; and greater mobilization of private capital for responsible value-chain development.
+MDBs will build a shared evidence base on their collective engagement in critical minerals value chains. An annual stocktake will track agreed high-level information, which will include countries and regions supported, value-chain segments, intervention types, technical assistance, financing, collaboration modalities, co-financed operations, and selected development results at aggregate level.
+The MDBs will also foster operational learning. MDBs will exchange lessons on policy reform, ESG application, corridor planning, infrastructure sequencing, local value addition, community engagement (including with CSOs) and benefit-sharing, project preparation, de-risking, financing instruments, and partnerships with public and private actors. Where feasible, participating institutions may undertake joint evaluations of selected operations using common questions or indicators.
+The intended result is greater transparency, a clearer understanding of gaps and opportunities, better- targeted collaboration, stronger accountability to MDB leadership and partners, and faster replication of approaches that demonstrate results.
+1 The Framework does not restrict the ability of governments and the private sector clients to engage with, or see support from, the MDB or combination of MDBs of their choice. Participation in any collaborative arrangement will remain subject to the client’s agreement.</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:10:11.473153+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>EBRD support to boost growth for Türkiye’s Sanmar</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-support-to-boost-growth-for-tuerkiye-s-sanmar.html</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+The European Bank for Reconstruction and Development (EBRD) is providing €22.5 million to Sanmar Denizcilik Makina ve Ticaret (Sanmar), one of the world’s leading tugboat manufacturers, to support the company's growth and green transition.
+The financing comes as part of a risk-sharing facility between the EBRD and Akbank, strengthening the two institutions’ partnership in supporting sustainable investment and industrial development in Türkiye, with a particular focus on small and medium-sized enterprises (SMEs) and mid-cap companies.
+The proceeds will help Sanmar to meet working capital requirements as it expands production and delivery of fully electric tugboats, supporting the company’s growth in an increasingly decarbonised maritime sector. The overall financing package amounts to €45 million, including a €5 million uncommitted tranche to support the installation of a 5 MW solar photovoltaic power plant for Sanmar’s own electricity consumption.
+Founded in 1976, Sanmar is a pioneering Turkish shipbuilder with a long track record of innovation in the maritime sector. The company has delivered several global industry firsts, including the world's first liquefied natural gas (LNG)-fuelled tugboats, the world's first remotely operated commercial vessel, Europe’s first electric tugboat, the world’s first methanol-fuelled tugboats and the world’s first transverse tugboat.
+İdil Gürsel, EBRD Deputy Head of Türkiye, said: “Türkiye continues to demonstrate its strength as a centre for industrial innovation and green investment. Through our partnership with Sanmar and Akbank, we are supporting the development of cutting-edge electric maritime technologies while helping to advance the decarbonisation of the shipping sector. This project combines competitiveness, innovation and climate action, fully reflecting the EBRD’s priorities in Türkiye.”
+Ali Gürün, Chairman of the Board of Sanmar, said: “Sanmar’s long-standing environmental, social and governance commitment has enabled us to meet the high standards required for this important financing partnership with the EBRD and Akbank. This support will further strengthen our investment in sustainable shipbuilding and accelerate our contribution to the maritime industry’s transition towards a cleaner, low-carbon future.”
+Akbank Executive Vice President of Commercial Banking Özlem Atik said: “At Akbank, we attach great importance to facilitating our customers’ access to the financing they need throughout their growth and investment journeys, and to leveraging our strong partnerships with international financial institutions for the benefit of the real economy. The €45 million financing we have provided to Sanmar Denizcilik, one of the leading players in the maritime sector, together with the EBRD, is an important example of this approach. Going forward, we will continue to develop financing solutions that support our customers’ competitiveness and sustainable growth.”
+The project supports the decarbonisation of maritime transport by enabling the production and delivery of zero-direct-emission electric tugboats. According to project assessments, each vessel is expected to reduce greenhouse gas emissions by approximately 1,800 tonnes of CO₂ equivalent annually compared with conventional diesel-powered alternatives. The solar power installation is expected to avoid a further 2,600 tonnes of CO₂ emissions annually.
+The EBRD is one of Türkiye’s key investors, with more than €26 billion committed since 2009, largely in the private sector.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:10:15.740008+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>EBRD welcomes G7 commitment to finance urgent repairs to Chornobyl’s protective shield</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-welcomes-g7-commitment-to-finance-urgent-repairs-to-chornob.html</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+Author: Nigina Mirbabaeva
+The European Bank for Reconstruction and Development (EBRD) welcomes the announcement by the Group of Seven (G7)that as leading industrialised nations, they will provide €260 million to fund urgent repairs to the New Safe Confinement at the Chornobyl Nuclear Power Plant in Ukraine, following the Russian drone strike that severely damaged the structure in February 2025.
+The G7 (Canada, France, Germany, Italy, Japan, the United Kingdom and the United States) expressed grave concern over the nuclear safety risks caused by the strike and pledged to mobilise funding to repair the New Safe Confinement. The structure contains the remains of Reactor Four and enables the safe dismantling of the original containment sarcophagus built after the 1986 accident.
+The G7 also called on other international partners to join the effort and contribute to covering the remaining financing needs.
+The announcement was made at the International Monetary Fund and World Bank Autumn Meetings in Bangkok, following a meeting of the G7 finance ministers.
+EBRD President Odile Renaud-Basso said: “The EBRD is grateful to the G7 nations for their continued leadership and commitment to nuclear safety at Chornobyl. We join the G7 in calling on the wider international community to contribute to these efforts at a donor conference we are convening in Paris on 9 November 2026, co-chaired by France, Ukraine and the EBRD.”
+Chornobyl’s New Safe Confinement was severely damaged by a Russian drone strike on 14 February 2025. The attack breached the structure’s inner and outer cladding, damaged critical systems and severely compromised its two primary functions: containing radioactive material and enabling the safe dismantling of the unstable original sarcophagus over Reactor Four.
+Preliminary assessments indicate that at least €500 million will be needed to repair the damage and restore the structure to full functionality. The work needs to be completed by 2030 to limit the risk of corrosion of the steel arch and safeguard the structure’s 100-year design life.
+The EBRD has led global efforts to stabilise and manage risks at Chornobyl since 1995, mobilising over €2.5 billion in international contributions – much of it from the G7 nations – and providing more than €700 million of its own resources to fund nuclear safety and decommissioning projects linked to the site.
+The Bank is now leading international efforts to restore the full functionality of the New Safe Confinement and to mobilise the remaining funding needed for urgent repairs.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:10:18.493743+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Helping women entrepreneurs thrive across the southern and eastern Mediterranean</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/videos/2026/helping-women-entrepreneurs-thrive-across-the-southern-and-easte.html</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Helping women entrepreneurs thrive across the southern and eastern Mediterranean
+Access to finance and know-how helps women entrepreneurs turn ambition into thriving businesses, creating jobs and new opportunities in their communities.
+Women entrepreneurs across Egypt, Jordan, Morocco and Tunisia are growing their businesses and creating jobs with support from the EBRD and the European Union (EU).
+Through the Financial Inclusion Programme, access to finance and expert advice is helping entrepreneurs turn ambition into opportunity. Watch their stories to see how this support is strengthening businesses and communities across the southern and eastern Mediterranean region.
+Video for media use
+If you would like a broadcast-quality version of this or any other EBRD video, including B-roll, please contact our Communications Department.</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:10:21.666162+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>EBRD invests €40 million to support businesses in central and eastern Europe</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-invests--40-million-to-support-businesses-in-central-and-ea.html</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+Author: Nigina Mirbabaeva
+The European Bank for Reconstruction and Development (EBRD) has invested up to €40 million in Avallon MBO Fund IV, a private equity fund focused on supporting small and medium-sized enterprises (SMEs) and small mid-cap companies in Poland and elsewhere in central and eastern Europe.
+The investment will promote private enterprise, encourage management to take ownership stakes in their companies and help those businesses to build operational capacity, innovate and grow.
+Avallon MBO Fund IV, managed by Avallon, is targeting total commitments of €220 million, with a maximum size of €260 million. At least 70 per cent of the fund's commitments will be invested in Poland, with up to 30 per cent allocated elsewhere in central and eastern Europe, namely Bulgaria, Croatia, Czechia, Estonia, Hungary, Latvia, Lithuania, Romania, the Slovak Republic and Slovenia. The fund will build a diversified portfolio of equity and quasi-equity investments in SMEs and small mid-caps, providing long-term capital to help businesses scale up and become more competitive.
+The EBRD's participation will play a key role in mobilising additional investment and strengthening fundraising efforts in a market where access to long-term risk capital remains limited. Private equity fundraising across central and eastern Europe has faced challenges in recent years, affecting the availability of growth financing for smaller businesses.
+Andreea Moraru, Managing Director for Central Europe and the Baltic States at the EBRD, said: "Small and medium-sized companies are a vital source of innovation, employment and economic growth. Through our investment in Avallon MBO Fund IV, we will help ambitious businesses strengthen their market position, pursue new opportunities and contribute to sustainable economic development across the region."
+Dirk Werner, Managing Director for Equity at the EBRD, added: “With fundraising conditions remaining difficult even for established managers, the EBRD's support is instrumental in bringing in institutional-quality investors and strengthening the development of private equity funds, which are increasingly needed in today's environment.”
+Tomasz Stamirowski, Managing Partner of Avallon, said: “The EBRD has been a key investor in four consecutive funds. We value both our long-standing relationship and the enormous role the EBRD plays in the success of fundraising in central and eastern Europe.”
+Avallon is a Poland-based private equity manager with a focus on investing in SMEs and supporting their development across central and eastern Europe. For over 25 years, Avallon has worked with management teams to support companies through succession, expansion, professionalisation and market consolidation.
+The EBRD is one of the leading institutional investors in Poland, having invested more than €17 billion in the country across more than 610 projects to date. It finances companies at every stage of growth through debt, equity and equity-like instruments both directly and indirectly. 
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:10:25.969271+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>EBRD makes €99.1 million loan to modernise mining sector in Côte d’Ivoire and Senegal</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-makes--99-1-million-loan-to-modernise-mining-sector-in-cote.html</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+The European Bank for Reconstruction and Development (EBRD) is providing a €99.1 million (US$ 111 million equivalent) loan to Mota-Engil Africa to support mining services operations in Côte d’Ivoire and Senegal.
+Mota-Engil Africa is one of Africa's leading engineering, construction and mining services companies, and works on major mining and infrastructure projects across the continent.
+The EBRD's investment will help finance purchases of modern equipment, support working capital requirements and refinance recent investments at three mines in Côte d’Ivoire and Senegal. This will help improve productivity, strengthen operational capacity and enhance the sustainability of mining operations.
+Replacing older equipment with newer, more environmentally friendly machinery will lower fuel consumption and reduce greenhouse gas emissions.
+As part of the EBRD agreement, Mota-Engil Africa will also make a strategic investment in developing local human capital. This will include enhancing the skills of its workforce and establishing nationally accredited technical training programmes in partnership with educational institutions in Côte d’Ivoire and Senegal. The programmes will equip participants with the technical skills required by the modern mining industry, strengthen the pipeline of qualified talent and expand access to quality employment opportunities.Mota-Engil Africa will also implement targeted measures to increase women’s participation across the sector, including initiatives to recruit, retain and advance women in technical, operational and leadership positions.
+Both workstreams will be supported by a €200,000 technical cooperation programme provided by the EBRD under its Gender and Economic Inclusion Framework.
+The EBRD began investing in sub-Saharan Africa in 2025. The Bank has so far invested more than €620 million across Benin , Côte d’Ivoire, Kenya , Nigeria and Senegal , supporting private-sector growth, financial institutions, infrastructure, energy, natural resources, telecommunications and agribusiness.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:10:30.148166+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Safe water, better lives in the Kyrgyz Republic</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/videos/2026/safe-water--better-lives-in-the-kyrgyz-republic.html</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Safe water, better lives in the Kyrgyz Republic
+Safe drinking water means better health, a more reliable daily life and a brighter future for communities across the Kyrgyz Republic.
+Access to safe drinking water is changing lives across the Kyrgyz Republic. EBRD investments have helped nearly 3 million people benefit from safe water and improved services.
+With support from the European Union (EU) and other international donors, these projects are helping build healthier, more resilient communities. Watch our video to see the difference reliable water services make to people’s everyday lives.
+Video for media use
+If you would like a broadcast-quality version of this or any other EBRD video, including B-roll, please contact our Communications Department.</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:10:33.330666+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>EBRD finances rehabilitation of Moldova’s key irrigation systems</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-finances-rehabilitation-of-moldova-s-key-irrigation-systems.html</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>EBRD supports growth of Auto Rubber in Uzbekistan
+Project to help transform company into a diversified automotive component manufacturer
+30 Oct 2026
+Who we are
+Overview: about the EBRD
+Explore the EBRD’s journey over the decades, investing in businesses, supporting economies and driving lasting change across its regions.
+What we do
+Overview: how the EBRD operates
+Across three continents, the EBRD supports the transition to successful market economies.
+Work with us
+Overview: how you can work with the EBRD
+We draw on three decades of regional knowledge and financial expertise to tailor our products and approaches to each client's needs.
+Author: Nigina Mirbabaeva
+The European Bank for Reconstruction and Development (EBRD) is lending €102.9 million to the government of Moldova to finance the rehabilitation and modernisation of priority centralised irrigation systems. The Bank’s investment will help restore reliable irrigation services, improve agricultural water security and build a more resilient and competitive agricultural sector in Moldova.
+Up to €49.8 million of the EBRD loan will finance the rehabilitation of the Puhacenii de Sus and Masivul Causeni centralised irrigation systems in the Nistru River basin, through the procurement and installation of modern water-intake, pumping and distribution infrastructure. This will restore reliable irrigation services to approximately 6,900 hectares of agricultural land where existing irrigation infrastructure is obsolete, non-functional or underutilised.
+This will also be complemented by an investment grant of €4.8 million from the European Union (EU) Neighbourhood Investment Platform and a national contribution of up to €7.2 million under the EU Growth Plan for Moldova.
+The remaining loan amount of up to €53.1 million will finance the rehabilitation of additional priority centralised irrigation systems, to be identified by the government.
+Together, these investments will help modernise Moldova’s irrigation infrastructure, reduce farmers’ exposure to climate-related production shocks and support a gradual transition towards more reliable, sustainable and higher-value agricultural production.
+Modernised systems such as pressurised pipe networks, appropriately sized pumping equipment, variable-speed drives and automated controls are expected to lead to more energy-efficient water distribution, saving around 13 million cubic metres of water a year, while supporting a threefold increase in annual agricultural output in the rehabilitated areas.
+The investment also aims to strengthen the capacity of Moldova’s National Agency for Land Improvement as the project implementation unit, and to enable water users’ associations and farmers to manage and maintain the systems sustainably. Technical assistance will support asset management, financial planning, service-fee setting and digital reporting, as well as measures to increase the participation of women and young farmers in irrigation governance and training.
+The EBRD is Moldova’s biggest institutional investor. Since the start of Russia’s full-scale invasion of neighbouring Ukraine, the Bank has provided €1.7 billion to Moldova to help mitigate the economic consequences of the war on the country’s economy. Overall, the Bank has invested more than €3.1 billion across 201 projects in the country.
+About the EU Growth Plan
+The Growth Plan for the Republic of Moldova, worth €1.9 billion for 2025-27, is the largest EU financial support package provided to Moldova since the country’s independence. It will boost Moldova’s economy, bring the country closer to EU membership by accelerating reforms, enhance access to the EU’s single market and provide significant financial assistance through a dedicated Reform and Growth Facility for Moldova. The Growth Plan will mobilise investments for jobs and growth and, most importantly, transform the lives of Moldovan citizens.
+Funds to support growth at the fast-moving consumer goods retailer
+New €87 million to deliver more sustainable and resilient urban infrastructure in 15 countries</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:10:37.315700+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily news scrape: 2026-10-31
</commit_message>
<xml_diff>
--- a/EBRD.xlsx
+++ b/EBRD.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -4696,6 +4696,49 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>EBRD arranges US$ 265 million loan for ADD Properties in Egypt</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>https://www.ebrd.com/content/ebrd_dxp/uk/en/home/news-and-events/news/2026/ebrd-arranges-us--265-million-loan-for-add-properties-in-egypt.html</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>EBRD arranges US$ 265 million loan for ADD Properties in Egypt
+EBRD, IFC, Emirates NBD Group and National Bank of Egypt join forces to support sustainable tourism-sector growth
+30 Oct 2026
+The European Bank for Reconstruction and Development (EBRD) is arranging a US$ 265 million financing package to support the expansion and modernisation of the hospitality operations of ADD Properties, a member of Sami Saad Holding, in Egypt.
+The EBRD has been mandated as the initial lead arranger (IMLA) and bookrunner, and is providing the largest facility, at US$ 127.5 million. The International Finance Corporation (IFC), acting as a mandated lead arranger (MLA) is extending a loan of US$ 60 million by way of the Mutual Reliance Framework.
+Emirates NBD Egypt is acting as MLA, global facility agent and onshore account bank, providing US$ 40 million. DenizBank AG, a subsidiary of Emirates NBD Group, is serving as the offshore security agent and offshore account bank. National Bank of Egypt, acting as MLA, local facility agent and onshore security agent, as well as the onshore account bank, is providing a US$ 37.5 million loan. EFG Hermes, an EFG Holding company, is acting as the sole financial advisor and bookrunner on the transaction.
+The financing aims to strengthen ADD Properties’ capital structure ADD Properties - Member of Sami Saad Holding, support the continued growth and enhancement of its hospitality portfolio, and consolidate its asset value in a period of significant capital deployment, anchored by the development of a new Grand Hyatt hotel in West Cairo.
+ADD Properties’ expansion reinforces Egypt’s national tourism strategy and enhances the hospitality offering in one of the country’s fastest-growing destinations, where cultural and leisure tourism are surging, driven by the opening of the Grand Egyptian Museum and ongoing regeneration of the Giza Plateau.
+Bassel Sami Saad, Chairman of ADD Properties, said: “This partnership reflects the confidence of leading international and regional financial institutions in Egypt’s investment potential and ADD Properties’ long-term vision. Together with our partners, we are advancing sustainable hospitality and branded residence development, in alignment with Egypt Vision 2030. Our new Grand Hyatt overlooking the Grand Egyptian Museum and the Pyramids of Giza embodies our ambition to create lasting value while celebrating Egypt’s extraordinary heritage.”
+Vlaho Kojakovic, EBRD Director for Real Estate, said: “Egypt’s tourism sector has significant potential to drive investment, job creation and sustainable economic growth. This financing reflects the strength of the partnership between the EBRD and ADD Properties, and our shared ambition to support the long-term development of a more sustainable and competitive tourism sector in Egypt. By supporting ADD Properties’ continued growth and investment in high-quality hospitality infrastructure, including the new Grand Hyatt in West Cairo, we are helping to strengthen Egypt’s tourism offering while promoting higher standards in sustainability, skills and corporate governance. We look forward to building on this partnership as ADD Properties continues to grow and invest in Egypt’s tourism sector.”
+Ary Naïm, IFC Division Director for North Africa and the Horn of Africa said: “The tourism industry is a powerful engine for job creation and economic development globally, and Egypt has great potential to better leverage its unique cultural and natural assets towards these goals. Our financing, in partnership with EBRD and others, will support ADD Properties to expand and upgrade its capacity while building sustainability and resilience, creating opportunities for local businesses and communities, and mobilizing private capital.”
+Amr ElShafei, Chief Executive Officer and Managing Director of Emirates NBD Egypt, said: “Our participation in this landmark financing reflects Emirates NBD Group’s strong commitment to supporting Egypt’s economic growth and to advancing the development of its strategic real-estate and hospitality sectors. We are proud to support ADD Properties, a prominent real-estate and hospitality developer, in advancing its growth strategy. Emirates NBD Egypt, alongside DenizBank AG, will bring together the strength of our regional banking franchise and our international capabilities to support a complex, large-scale financing transaction. Our collaboration with the EBRD, the IFC and National Bank of Egypt demonstrates the value of strong banking partnerships supporting high-quality investments.”
+Mohamed El-Etreby, Chief Executive Officer of National Bank of Egypt, said: “This long-term syndicated facility reflects National Bank of Egypt’s commitment to supporting strategic industries, particularly tourism, which is a vital pillar of the Egyptian economy and a key driver of sustainable growth, increasing foreign-currency proceeds and creating job opportunities. This strategic financing consortium reflects our commitment to fostering strategic partnerships with leading international financial institutions to support high-impact projects that contribute to strengthening Egypt’s position as a leading global tourism destination.”
+The financing will be complemented by technical assistance to deliver inclusive, green and market-relevant training programmes for young women and men in Cairo and Hurghada, strengthening the supply of skilled labour in Egypt’s hospitality sector.
+Technical assistance will support improvements in corporate governance, with the implementation of a corporate governance action plan aimed at strengthening ADD Properties’ governance practices. The assistance will further support a portfolio-wide green transition, including the development of a high-performance hotel and the certification of existing assets to LEED “Silver” standards.
+Through this investment, the EBRD reaffirms its commitment to supporting Egypt’s tourism sector, fostering sustainable growth and enhancing the quality and resilience of hospitality infrastructure.
+Egypt is a founding member of the EBRD. Since 2012, the Bank has invested more than €16 billion in 238 projects across the country.</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2026-10-31T10:42:12.985144+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>